<commit_message>
Evaluación prácticas 1 y 2
</commit_message>
<xml_diff>
--- a/Evaluacion.xlsx
+++ b/Evaluacion.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uo295526\git\alg_GisbertLucasUO295526\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\user2\juanrp\git\alg2024\alg_GisbertLucasUO295526\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -15,21 +15,11 @@
     <sheet name="Marks" sheetId="4" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Estudiante</t>
   </si>
@@ -98,6 +88,18 @@
   </si>
   <si>
     <t>https://github.com/uo295526/alg_GisbertLucasUO295526</t>
+  </si>
+  <si>
+    <t>No aparece ninguna identificación en el documento. No se numeran las páginas. P0. Las gráficas mejor junto a las tablas y mejor copiarlas en formato vectorial para poder hacerlas más grandes sin que pierdan calidad. Las gráficas son incorrectas, deben representarse los valores de n correctamente. P11. De nuevo gráficas separadas e incorrectas. P12. Algunos tiempos no parece que estén correctamente medidos. Mismo comentario de las gráficas que para documentos anteriores.</t>
+  </si>
+  <si>
+    <t>R-</t>
+  </si>
+  <si>
+    <t>Documento sin identificación. Sería interesante numerar páginas. Tiempos parecen correctos. Representación correcta, pero fusionar en una misma gráfica para comparar las distintas posibilidades para un algortimo, salvo diferencias en la complejidad. Gráficas junto a la tabla de valores correspondiente.</t>
+  </si>
+  <si>
+    <t>B-</t>
   </si>
 </sst>
 </file>
@@ -107,10 +109,17 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -148,6 +157,29 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color indexed="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -157,7 +189,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -217,23 +249,102 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -242,13 +353,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -257,11 +368,78 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="64">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
+    <cellStyle name="Hipervínculo 2" xfId="3"/>
+    <cellStyle name="Hipervínculo 3" xfId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="5"/>
+    <cellStyle name="Normal 3" xfId="6"/>
+    <cellStyle name="Normal 3 2" xfId="7"/>
+    <cellStyle name="Normal 3 3" xfId="8"/>
+    <cellStyle name="Normal 3 4" xfId="9"/>
+    <cellStyle name="Normal 3 4 2" xfId="10"/>
+    <cellStyle name="Normal 3 4 2 2" xfId="11"/>
+    <cellStyle name="Normal 3 4 3" xfId="12"/>
+    <cellStyle name="Normal 3 5" xfId="13"/>
+    <cellStyle name="Normal 3 5 2" xfId="14"/>
+    <cellStyle name="Normal 4" xfId="15"/>
+    <cellStyle name="Normal 4 2" xfId="16"/>
+    <cellStyle name="Normal 4 2 2" xfId="17"/>
+    <cellStyle name="Normal 4 2 2 2" xfId="18"/>
+    <cellStyle name="Normal 4 2 2 2 2" xfId="19"/>
+    <cellStyle name="Normal 4 2 2 3" xfId="20"/>
+    <cellStyle name="Normal 4 2 3" xfId="21"/>
+    <cellStyle name="Normal 4 2 3 2" xfId="22"/>
+    <cellStyle name="Normal 4 2 4" xfId="23"/>
+    <cellStyle name="Normal 4 3" xfId="24"/>
+    <cellStyle name="Normal 4 3 2" xfId="25"/>
+    <cellStyle name="Normal 4 3 2 2" xfId="26"/>
+    <cellStyle name="Normal 4 3 3" xfId="27"/>
+    <cellStyle name="Normal 4 3 3 2" xfId="28"/>
+    <cellStyle name="Normal 4 3 4" xfId="29"/>
+    <cellStyle name="Normal 4 4" xfId="30"/>
+    <cellStyle name="Normal 4 4 2" xfId="31"/>
+    <cellStyle name="Normal 4 4 2 2" xfId="32"/>
+    <cellStyle name="Normal 4 4 3" xfId="33"/>
+    <cellStyle name="Normal 4 5" xfId="34"/>
+    <cellStyle name="Normal 4 5 2" xfId="35"/>
+    <cellStyle name="Normal 4 6" xfId="36"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
+    <cellStyle name="Porcentaje 2" xfId="37"/>
+    <cellStyle name="Porcentaje 2 2" xfId="38"/>
+    <cellStyle name="Porcentaje 2 3" xfId="39"/>
+    <cellStyle name="Porcentaje 2 3 2" xfId="40"/>
+    <cellStyle name="Porcentaje 2 3 2 2" xfId="41"/>
+    <cellStyle name="Porcentaje 2 3 3" xfId="42"/>
+    <cellStyle name="Porcentaje 2 4" xfId="43"/>
+    <cellStyle name="Porcentaje 2 4 2" xfId="44"/>
+    <cellStyle name="Porcentaje 3" xfId="45"/>
+    <cellStyle name="Porcentaje 4" xfId="46"/>
+    <cellStyle name="Porcentaje 4 2" xfId="47"/>
+    <cellStyle name="Porcentaje 4 3" xfId="48"/>
+    <cellStyle name="Porcentaje 4 4" xfId="49"/>
+    <cellStyle name="Porcentaje 4 4 2" xfId="50"/>
+    <cellStyle name="Porcentaje 4 4 2 2" xfId="51"/>
+    <cellStyle name="Porcentaje 4 4 3" xfId="52"/>
+    <cellStyle name="Porcentaje 4 5" xfId="53"/>
+    <cellStyle name="Porcentaje 4 5 2" xfId="54"/>
+    <cellStyle name="Porcentaje 5" xfId="55"/>
+    <cellStyle name="Porcentaje 5 2" xfId="56"/>
+    <cellStyle name="Porcentaje 5 2 2" xfId="57"/>
+    <cellStyle name="Porcentaje 5 3" xfId="58"/>
+    <cellStyle name="Porcentaje 6" xfId="59"/>
+    <cellStyle name="Porcentaje 6 2" xfId="60"/>
+    <cellStyle name="Porcentaje 7" xfId="61"/>
+    <cellStyle name="Porcentaje 7 2" xfId="62"/>
+    <cellStyle name="Porcentaje 8" xfId="63"/>
   </cellStyles>
   <dxfs count="20">
     <dxf>
@@ -984,14 +1162,22 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="100.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" ht="168.75" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
+      <c r="B5" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>26</v>
+      </c>
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>

</xml_diff>

<commit_message>
Revisión mezcla después de clase.
</commit_message>
<xml_diff>
--- a/Evaluacion.xlsx
+++ b/Evaluacion.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Estudiante</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>B-</t>
+  </si>
+  <si>
+    <t>Revisión mezcla después de clase. Implementación con muchos news. Junit en un main no funciona todavía. Clase tiempos.</t>
   </si>
 </sst>
 </file>
@@ -109,10 +112,17 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -265,86 +275,108 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="64">
+  <cellStyleXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -353,13 +385,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -368,14 +400,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="64">
+  <cellStyles count="86">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
     <cellStyle name="Hipervínculo 2" xfId="3"/>
     <cellStyle name="Hipervínculo 3" xfId="4"/>
@@ -395,23 +430,45 @@
     <cellStyle name="Normal 4 2 2" xfId="17"/>
     <cellStyle name="Normal 4 2 2 2" xfId="18"/>
     <cellStyle name="Normal 4 2 2 2 2" xfId="19"/>
+    <cellStyle name="Normal 4 2 2 2 2 2" xfId="68"/>
+    <cellStyle name="Normal 4 2 2 2 3" xfId="67"/>
     <cellStyle name="Normal 4 2 2 3" xfId="20"/>
+    <cellStyle name="Normal 4 2 2 3 2" xfId="69"/>
+    <cellStyle name="Normal 4 2 2 4" xfId="66"/>
     <cellStyle name="Normal 4 2 3" xfId="21"/>
     <cellStyle name="Normal 4 2 3 2" xfId="22"/>
+    <cellStyle name="Normal 4 2 3 2 2" xfId="71"/>
+    <cellStyle name="Normal 4 2 3 3" xfId="70"/>
     <cellStyle name="Normal 4 2 4" xfId="23"/>
+    <cellStyle name="Normal 4 2 4 2" xfId="72"/>
+    <cellStyle name="Normal 4 2 5" xfId="65"/>
     <cellStyle name="Normal 4 3" xfId="24"/>
     <cellStyle name="Normal 4 3 2" xfId="25"/>
     <cellStyle name="Normal 4 3 2 2" xfId="26"/>
+    <cellStyle name="Normal 4 3 2 2 2" xfId="75"/>
+    <cellStyle name="Normal 4 3 2 3" xfId="74"/>
     <cellStyle name="Normal 4 3 3" xfId="27"/>
     <cellStyle name="Normal 4 3 3 2" xfId="28"/>
+    <cellStyle name="Normal 4 3 3 2 2" xfId="77"/>
+    <cellStyle name="Normal 4 3 3 3" xfId="76"/>
     <cellStyle name="Normal 4 3 4" xfId="29"/>
+    <cellStyle name="Normal 4 3 4 2" xfId="78"/>
+    <cellStyle name="Normal 4 3 5" xfId="73"/>
     <cellStyle name="Normal 4 4" xfId="30"/>
     <cellStyle name="Normal 4 4 2" xfId="31"/>
     <cellStyle name="Normal 4 4 2 2" xfId="32"/>
+    <cellStyle name="Normal 4 4 2 2 2" xfId="81"/>
+    <cellStyle name="Normal 4 4 2 3" xfId="80"/>
     <cellStyle name="Normal 4 4 3" xfId="33"/>
+    <cellStyle name="Normal 4 4 3 2" xfId="82"/>
+    <cellStyle name="Normal 4 4 4" xfId="79"/>
     <cellStyle name="Normal 4 5" xfId="34"/>
     <cellStyle name="Normal 4 5 2" xfId="35"/>
+    <cellStyle name="Normal 4 5 2 2" xfId="84"/>
+    <cellStyle name="Normal 4 5 3" xfId="83"/>
     <cellStyle name="Normal 4 6" xfId="36"/>
+    <cellStyle name="Normal 4 6 2" xfId="85"/>
+    <cellStyle name="Normal 4 7" xfId="64"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
     <cellStyle name="Porcentaje 2" xfId="37"/>
     <cellStyle name="Porcentaje 2 2" xfId="38"/>
@@ -1178,7 +1235,9 @@
       <c r="E5" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="F5" s="17" t="s">
+        <v>27</v>
+      </c>
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>

</xml_diff>

<commit_message>
Evaluación hasta P6 backtracking
</commit_message>
<xml_diff>
--- a/Evaluacion.xlsx
+++ b/Evaluacion.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Estudiante</t>
   </si>
@@ -145,7 +145,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Tablas de tiempos incorrectas, tiempos por debajo del umbral. </t>
+      <t xml:space="preserve">Tablas de tiempos incorrectas, tiempos por debajo del umbral, nos indica que realmente este es el resultado después de medir repetidamente y aplicar el factor de conversión. </t>
     </r>
     <r>
       <rPr>
@@ -173,6 +173,12 @@
       <t>.</t>
     </r>
   </si>
+  <si>
+    <t>Test ok. Doc ok, indica patrones de dependencia en texto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestOne ok. Test5 1,19; test6 0,23; test7 36,7. </t>
+  </si>
 </sst>
 </file>
 
@@ -181,10 +187,17 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -357,74 +370,96 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="108">
+  <cellStyleXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
@@ -470,17 +505,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -489,13 +524,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -504,17 +539,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="108">
+  <cellStyles count="130">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
     <cellStyle name="Hipervínculo 2" xfId="3"/>
     <cellStyle name="Hipervínculo 3" xfId="4"/>
@@ -536,65 +580,87 @@
     <cellStyle name="Normal 4 2 2 2 2" xfId="19"/>
     <cellStyle name="Normal 4 2 2 2 2 2" xfId="68"/>
     <cellStyle name="Normal 4 2 2 2 2 3" xfId="90"/>
+    <cellStyle name="Normal 4 2 2 2 2 4" xfId="112"/>
     <cellStyle name="Normal 4 2 2 2 3" xfId="67"/>
     <cellStyle name="Normal 4 2 2 2 4" xfId="89"/>
+    <cellStyle name="Normal 4 2 2 2 5" xfId="111"/>
     <cellStyle name="Normal 4 2 2 3" xfId="20"/>
     <cellStyle name="Normal 4 2 2 3 2" xfId="69"/>
     <cellStyle name="Normal 4 2 2 3 3" xfId="91"/>
+    <cellStyle name="Normal 4 2 2 3 4" xfId="113"/>
     <cellStyle name="Normal 4 2 2 4" xfId="66"/>
     <cellStyle name="Normal 4 2 2 5" xfId="88"/>
+    <cellStyle name="Normal 4 2 2 6" xfId="110"/>
     <cellStyle name="Normal 4 2 3" xfId="21"/>
     <cellStyle name="Normal 4 2 3 2" xfId="22"/>
     <cellStyle name="Normal 4 2 3 2 2" xfId="71"/>
     <cellStyle name="Normal 4 2 3 2 3" xfId="93"/>
+    <cellStyle name="Normal 4 2 3 2 4" xfId="115"/>
     <cellStyle name="Normal 4 2 3 3" xfId="70"/>
     <cellStyle name="Normal 4 2 3 4" xfId="92"/>
+    <cellStyle name="Normal 4 2 3 5" xfId="114"/>
     <cellStyle name="Normal 4 2 4" xfId="23"/>
     <cellStyle name="Normal 4 2 4 2" xfId="72"/>
     <cellStyle name="Normal 4 2 4 3" xfId="94"/>
+    <cellStyle name="Normal 4 2 4 4" xfId="116"/>
     <cellStyle name="Normal 4 2 5" xfId="65"/>
     <cellStyle name="Normal 4 2 6" xfId="87"/>
+    <cellStyle name="Normal 4 2 7" xfId="109"/>
     <cellStyle name="Normal 4 3" xfId="24"/>
     <cellStyle name="Normal 4 3 2" xfId="25"/>
     <cellStyle name="Normal 4 3 2 2" xfId="26"/>
     <cellStyle name="Normal 4 3 2 2 2" xfId="75"/>
     <cellStyle name="Normal 4 3 2 2 3" xfId="97"/>
+    <cellStyle name="Normal 4 3 2 2 4" xfId="119"/>
     <cellStyle name="Normal 4 3 2 3" xfId="74"/>
     <cellStyle name="Normal 4 3 2 4" xfId="96"/>
+    <cellStyle name="Normal 4 3 2 5" xfId="118"/>
     <cellStyle name="Normal 4 3 3" xfId="27"/>
     <cellStyle name="Normal 4 3 3 2" xfId="28"/>
     <cellStyle name="Normal 4 3 3 2 2" xfId="77"/>
     <cellStyle name="Normal 4 3 3 2 3" xfId="99"/>
+    <cellStyle name="Normal 4 3 3 2 4" xfId="121"/>
     <cellStyle name="Normal 4 3 3 3" xfId="76"/>
     <cellStyle name="Normal 4 3 3 4" xfId="98"/>
+    <cellStyle name="Normal 4 3 3 5" xfId="120"/>
     <cellStyle name="Normal 4 3 4" xfId="29"/>
     <cellStyle name="Normal 4 3 4 2" xfId="78"/>
     <cellStyle name="Normal 4 3 4 3" xfId="100"/>
+    <cellStyle name="Normal 4 3 4 4" xfId="122"/>
     <cellStyle name="Normal 4 3 5" xfId="73"/>
     <cellStyle name="Normal 4 3 6" xfId="95"/>
+    <cellStyle name="Normal 4 3 7" xfId="117"/>
     <cellStyle name="Normal 4 4" xfId="30"/>
     <cellStyle name="Normal 4 4 2" xfId="31"/>
     <cellStyle name="Normal 4 4 2 2" xfId="32"/>
     <cellStyle name="Normal 4 4 2 2 2" xfId="81"/>
     <cellStyle name="Normal 4 4 2 2 3" xfId="103"/>
+    <cellStyle name="Normal 4 4 2 2 4" xfId="125"/>
     <cellStyle name="Normal 4 4 2 3" xfId="80"/>
     <cellStyle name="Normal 4 4 2 4" xfId="102"/>
+    <cellStyle name="Normal 4 4 2 5" xfId="124"/>
     <cellStyle name="Normal 4 4 3" xfId="33"/>
     <cellStyle name="Normal 4 4 3 2" xfId="82"/>
     <cellStyle name="Normal 4 4 3 3" xfId="104"/>
+    <cellStyle name="Normal 4 4 3 4" xfId="126"/>
     <cellStyle name="Normal 4 4 4" xfId="79"/>
     <cellStyle name="Normal 4 4 5" xfId="101"/>
+    <cellStyle name="Normal 4 4 6" xfId="123"/>
     <cellStyle name="Normal 4 5" xfId="34"/>
     <cellStyle name="Normal 4 5 2" xfId="35"/>
     <cellStyle name="Normal 4 5 2 2" xfId="84"/>
     <cellStyle name="Normal 4 5 2 3" xfId="106"/>
+    <cellStyle name="Normal 4 5 2 4" xfId="128"/>
     <cellStyle name="Normal 4 5 3" xfId="83"/>
     <cellStyle name="Normal 4 5 4" xfId="105"/>
+    <cellStyle name="Normal 4 5 5" xfId="127"/>
     <cellStyle name="Normal 4 6" xfId="36"/>
     <cellStyle name="Normal 4 6 2" xfId="85"/>
     <cellStyle name="Normal 4 6 3" xfId="107"/>
+    <cellStyle name="Normal 4 6 4" xfId="129"/>
     <cellStyle name="Normal 4 7" xfId="64"/>
     <cellStyle name="Normal 4 8" xfId="86"/>
+    <cellStyle name="Normal 4 9" xfId="108"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
     <cellStyle name="Porcentaje 2" xfId="37"/>
     <cellStyle name="Porcentaje 2 2" xfId="38"/>
@@ -1367,16 +1433,24 @@
       <c r="G5" s="16">
         <v>8</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="17">
-        <v>4</v>
-      </c>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
+      <c r="I5" s="20">
+        <v>7</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="19">
+        <v>7</v>
+      </c>
+      <c r="L5" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="M5" s="20">
+        <v>6</v>
+      </c>
       <c r="N5" s="9"/>
       <c r="O5" s="9"/>
       <c r="P5" s="9"/>

</xml_diff>

<commit_message>
Evaluación continua prácticas nota final sobre 7
</commit_message>
<xml_diff>
--- a/Evaluacion.xlsx
+++ b/Evaluacion.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Estudiante</t>
   </si>
@@ -179,6 +179,15 @@
   <si>
     <t xml:space="preserve">TestOne ok. Test5 1,19; test6 0,23; test7 36,7. </t>
   </si>
+  <si>
+    <t>Funciona test00</t>
+  </si>
+  <si>
+    <t>Superada 19:13</t>
+  </si>
+  <si>
+    <t>Sobre 7</t>
+  </si>
 </sst>
 </file>
 
@@ -187,10 +196,17 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -294,7 +310,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -369,196 +385,307 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="130">
+  <cellStyleXfs count="219">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="130">
+  <cellStyles count="219">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
     <cellStyle name="Hipervínculo 2" xfId="3"/>
     <cellStyle name="Hipervínculo 3" xfId="4"/>
@@ -574,93 +701,181 @@
     <cellStyle name="Normal 3 5" xfId="13"/>
     <cellStyle name="Normal 3 5 2" xfId="14"/>
     <cellStyle name="Normal 4" xfId="15"/>
+    <cellStyle name="Normal 4 10" xfId="130"/>
     <cellStyle name="Normal 4 2" xfId="16"/>
     <cellStyle name="Normal 4 2 2" xfId="17"/>
     <cellStyle name="Normal 4 2 2 2" xfId="18"/>
     <cellStyle name="Normal 4 2 2 2 2" xfId="19"/>
     <cellStyle name="Normal 4 2 2 2 2 2" xfId="68"/>
+    <cellStyle name="Normal 4 2 2 2 2 2 2" xfId="135"/>
     <cellStyle name="Normal 4 2 2 2 2 3" xfId="90"/>
+    <cellStyle name="Normal 4 2 2 2 2 3 2" xfId="136"/>
     <cellStyle name="Normal 4 2 2 2 2 4" xfId="112"/>
+    <cellStyle name="Normal 4 2 2 2 2 4 2" xfId="137"/>
+    <cellStyle name="Normal 4 2 2 2 2 5" xfId="134"/>
     <cellStyle name="Normal 4 2 2 2 3" xfId="67"/>
+    <cellStyle name="Normal 4 2 2 2 3 2" xfId="138"/>
     <cellStyle name="Normal 4 2 2 2 4" xfId="89"/>
+    <cellStyle name="Normal 4 2 2 2 4 2" xfId="139"/>
     <cellStyle name="Normal 4 2 2 2 5" xfId="111"/>
+    <cellStyle name="Normal 4 2 2 2 5 2" xfId="140"/>
+    <cellStyle name="Normal 4 2 2 2 6" xfId="133"/>
     <cellStyle name="Normal 4 2 2 3" xfId="20"/>
     <cellStyle name="Normal 4 2 2 3 2" xfId="69"/>
+    <cellStyle name="Normal 4 2 2 3 2 2" xfId="142"/>
     <cellStyle name="Normal 4 2 2 3 3" xfId="91"/>
+    <cellStyle name="Normal 4 2 2 3 3 2" xfId="143"/>
     <cellStyle name="Normal 4 2 2 3 4" xfId="113"/>
+    <cellStyle name="Normal 4 2 2 3 4 2" xfId="144"/>
+    <cellStyle name="Normal 4 2 2 3 5" xfId="141"/>
     <cellStyle name="Normal 4 2 2 4" xfId="66"/>
+    <cellStyle name="Normal 4 2 2 4 2" xfId="145"/>
     <cellStyle name="Normal 4 2 2 5" xfId="88"/>
+    <cellStyle name="Normal 4 2 2 5 2" xfId="146"/>
     <cellStyle name="Normal 4 2 2 6" xfId="110"/>
+    <cellStyle name="Normal 4 2 2 6 2" xfId="147"/>
+    <cellStyle name="Normal 4 2 2 7" xfId="132"/>
     <cellStyle name="Normal 4 2 3" xfId="21"/>
     <cellStyle name="Normal 4 2 3 2" xfId="22"/>
     <cellStyle name="Normal 4 2 3 2 2" xfId="71"/>
+    <cellStyle name="Normal 4 2 3 2 2 2" xfId="150"/>
     <cellStyle name="Normal 4 2 3 2 3" xfId="93"/>
+    <cellStyle name="Normal 4 2 3 2 3 2" xfId="151"/>
     <cellStyle name="Normal 4 2 3 2 4" xfId="115"/>
+    <cellStyle name="Normal 4 2 3 2 4 2" xfId="152"/>
+    <cellStyle name="Normal 4 2 3 2 5" xfId="149"/>
     <cellStyle name="Normal 4 2 3 3" xfId="70"/>
+    <cellStyle name="Normal 4 2 3 3 2" xfId="153"/>
     <cellStyle name="Normal 4 2 3 4" xfId="92"/>
+    <cellStyle name="Normal 4 2 3 4 2" xfId="154"/>
     <cellStyle name="Normal 4 2 3 5" xfId="114"/>
+    <cellStyle name="Normal 4 2 3 5 2" xfId="155"/>
+    <cellStyle name="Normal 4 2 3 6" xfId="148"/>
     <cellStyle name="Normal 4 2 4" xfId="23"/>
     <cellStyle name="Normal 4 2 4 2" xfId="72"/>
+    <cellStyle name="Normal 4 2 4 2 2" xfId="157"/>
     <cellStyle name="Normal 4 2 4 3" xfId="94"/>
+    <cellStyle name="Normal 4 2 4 3 2" xfId="158"/>
     <cellStyle name="Normal 4 2 4 4" xfId="116"/>
+    <cellStyle name="Normal 4 2 4 4 2" xfId="159"/>
+    <cellStyle name="Normal 4 2 4 5" xfId="156"/>
     <cellStyle name="Normal 4 2 5" xfId="65"/>
+    <cellStyle name="Normal 4 2 5 2" xfId="160"/>
     <cellStyle name="Normal 4 2 6" xfId="87"/>
+    <cellStyle name="Normal 4 2 6 2" xfId="161"/>
     <cellStyle name="Normal 4 2 7" xfId="109"/>
+    <cellStyle name="Normal 4 2 7 2" xfId="162"/>
+    <cellStyle name="Normal 4 2 8" xfId="131"/>
     <cellStyle name="Normal 4 3" xfId="24"/>
     <cellStyle name="Normal 4 3 2" xfId="25"/>
     <cellStyle name="Normal 4 3 2 2" xfId="26"/>
     <cellStyle name="Normal 4 3 2 2 2" xfId="75"/>
+    <cellStyle name="Normal 4 3 2 2 2 2" xfId="166"/>
     <cellStyle name="Normal 4 3 2 2 3" xfId="97"/>
+    <cellStyle name="Normal 4 3 2 2 3 2" xfId="167"/>
     <cellStyle name="Normal 4 3 2 2 4" xfId="119"/>
+    <cellStyle name="Normal 4 3 2 2 4 2" xfId="168"/>
+    <cellStyle name="Normal 4 3 2 2 5" xfId="165"/>
     <cellStyle name="Normal 4 3 2 3" xfId="74"/>
+    <cellStyle name="Normal 4 3 2 3 2" xfId="169"/>
     <cellStyle name="Normal 4 3 2 4" xfId="96"/>
+    <cellStyle name="Normal 4 3 2 4 2" xfId="170"/>
     <cellStyle name="Normal 4 3 2 5" xfId="118"/>
+    <cellStyle name="Normal 4 3 2 5 2" xfId="171"/>
+    <cellStyle name="Normal 4 3 2 6" xfId="164"/>
     <cellStyle name="Normal 4 3 3" xfId="27"/>
     <cellStyle name="Normal 4 3 3 2" xfId="28"/>
     <cellStyle name="Normal 4 3 3 2 2" xfId="77"/>
+    <cellStyle name="Normal 4 3 3 2 2 2" xfId="174"/>
     <cellStyle name="Normal 4 3 3 2 3" xfId="99"/>
+    <cellStyle name="Normal 4 3 3 2 3 2" xfId="175"/>
     <cellStyle name="Normal 4 3 3 2 4" xfId="121"/>
+    <cellStyle name="Normal 4 3 3 2 4 2" xfId="176"/>
+    <cellStyle name="Normal 4 3 3 2 5" xfId="173"/>
     <cellStyle name="Normal 4 3 3 3" xfId="76"/>
+    <cellStyle name="Normal 4 3 3 3 2" xfId="177"/>
     <cellStyle name="Normal 4 3 3 4" xfId="98"/>
+    <cellStyle name="Normal 4 3 3 4 2" xfId="178"/>
     <cellStyle name="Normal 4 3 3 5" xfId="120"/>
+    <cellStyle name="Normal 4 3 3 5 2" xfId="179"/>
+    <cellStyle name="Normal 4 3 3 6" xfId="172"/>
     <cellStyle name="Normal 4 3 4" xfId="29"/>
     <cellStyle name="Normal 4 3 4 2" xfId="78"/>
+    <cellStyle name="Normal 4 3 4 2 2" xfId="181"/>
     <cellStyle name="Normal 4 3 4 3" xfId="100"/>
+    <cellStyle name="Normal 4 3 4 3 2" xfId="182"/>
     <cellStyle name="Normal 4 3 4 4" xfId="122"/>
+    <cellStyle name="Normal 4 3 4 4 2" xfId="183"/>
+    <cellStyle name="Normal 4 3 4 5" xfId="180"/>
     <cellStyle name="Normal 4 3 5" xfId="73"/>
+    <cellStyle name="Normal 4 3 5 2" xfId="184"/>
     <cellStyle name="Normal 4 3 6" xfId="95"/>
+    <cellStyle name="Normal 4 3 6 2" xfId="185"/>
     <cellStyle name="Normal 4 3 7" xfId="117"/>
+    <cellStyle name="Normal 4 3 7 2" xfId="186"/>
+    <cellStyle name="Normal 4 3 8" xfId="163"/>
     <cellStyle name="Normal 4 4" xfId="30"/>
     <cellStyle name="Normal 4 4 2" xfId="31"/>
     <cellStyle name="Normal 4 4 2 2" xfId="32"/>
     <cellStyle name="Normal 4 4 2 2 2" xfId="81"/>
+    <cellStyle name="Normal 4 4 2 2 2 2" xfId="190"/>
     <cellStyle name="Normal 4 4 2 2 3" xfId="103"/>
+    <cellStyle name="Normal 4 4 2 2 3 2" xfId="191"/>
     <cellStyle name="Normal 4 4 2 2 4" xfId="125"/>
+    <cellStyle name="Normal 4 4 2 2 4 2" xfId="192"/>
+    <cellStyle name="Normal 4 4 2 2 5" xfId="189"/>
     <cellStyle name="Normal 4 4 2 3" xfId="80"/>
+    <cellStyle name="Normal 4 4 2 3 2" xfId="193"/>
     <cellStyle name="Normal 4 4 2 4" xfId="102"/>
+    <cellStyle name="Normal 4 4 2 4 2" xfId="194"/>
     <cellStyle name="Normal 4 4 2 5" xfId="124"/>
+    <cellStyle name="Normal 4 4 2 5 2" xfId="195"/>
+    <cellStyle name="Normal 4 4 2 6" xfId="188"/>
     <cellStyle name="Normal 4 4 3" xfId="33"/>
     <cellStyle name="Normal 4 4 3 2" xfId="82"/>
+    <cellStyle name="Normal 4 4 3 2 2" xfId="197"/>
     <cellStyle name="Normal 4 4 3 3" xfId="104"/>
+    <cellStyle name="Normal 4 4 3 3 2" xfId="198"/>
     <cellStyle name="Normal 4 4 3 4" xfId="126"/>
+    <cellStyle name="Normal 4 4 3 4 2" xfId="199"/>
+    <cellStyle name="Normal 4 4 3 5" xfId="196"/>
     <cellStyle name="Normal 4 4 4" xfId="79"/>
+    <cellStyle name="Normal 4 4 4 2" xfId="200"/>
     <cellStyle name="Normal 4 4 5" xfId="101"/>
+    <cellStyle name="Normal 4 4 5 2" xfId="201"/>
     <cellStyle name="Normal 4 4 6" xfId="123"/>
+    <cellStyle name="Normal 4 4 6 2" xfId="202"/>
+    <cellStyle name="Normal 4 4 7" xfId="187"/>
     <cellStyle name="Normal 4 5" xfId="34"/>
     <cellStyle name="Normal 4 5 2" xfId="35"/>
     <cellStyle name="Normal 4 5 2 2" xfId="84"/>
+    <cellStyle name="Normal 4 5 2 2 2" xfId="205"/>
     <cellStyle name="Normal 4 5 2 3" xfId="106"/>
+    <cellStyle name="Normal 4 5 2 3 2" xfId="206"/>
     <cellStyle name="Normal 4 5 2 4" xfId="128"/>
+    <cellStyle name="Normal 4 5 2 4 2" xfId="207"/>
+    <cellStyle name="Normal 4 5 2 5" xfId="204"/>
     <cellStyle name="Normal 4 5 3" xfId="83"/>
+    <cellStyle name="Normal 4 5 3 2" xfId="208"/>
     <cellStyle name="Normal 4 5 4" xfId="105"/>
+    <cellStyle name="Normal 4 5 4 2" xfId="209"/>
     <cellStyle name="Normal 4 5 5" xfId="127"/>
+    <cellStyle name="Normal 4 5 5 2" xfId="210"/>
+    <cellStyle name="Normal 4 5 6" xfId="203"/>
     <cellStyle name="Normal 4 6" xfId="36"/>
     <cellStyle name="Normal 4 6 2" xfId="85"/>
+    <cellStyle name="Normal 4 6 2 2" xfId="212"/>
     <cellStyle name="Normal 4 6 3" xfId="107"/>
+    <cellStyle name="Normal 4 6 3 2" xfId="213"/>
     <cellStyle name="Normal 4 6 4" xfId="129"/>
+    <cellStyle name="Normal 4 6 4 2" xfId="214"/>
+    <cellStyle name="Normal 4 6 5" xfId="211"/>
     <cellStyle name="Normal 4 7" xfId="64"/>
+    <cellStyle name="Normal 4 7 2" xfId="215"/>
     <cellStyle name="Normal 4 8" xfId="86"/>
+    <cellStyle name="Normal 4 8 2" xfId="216"/>
     <cellStyle name="Normal 4 9" xfId="108"/>
+    <cellStyle name="Normal 4 9 2" xfId="217"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
     <cellStyle name="Porcentaje 2" xfId="37"/>
     <cellStyle name="Porcentaje 2 2" xfId="38"/>
@@ -689,6 +904,7 @@
     <cellStyle name="Porcentaje 7" xfId="61"/>
     <cellStyle name="Porcentaje 7 2" xfId="62"/>
     <cellStyle name="Porcentaje 8" xfId="63"/>
+    <cellStyle name="Porcentaje 8 2" xfId="218"/>
   </cellStyles>
   <dxfs count="20">
     <dxf>
@@ -1415,192 +1631,202 @@
       <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="15">
         <v>7</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="17">
+      <c r="E5" s="15">
         <v>8</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="14">
         <v>8</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="20">
+      <c r="I5" s="18">
         <v>7</v>
       </c>
-      <c r="J5" s="18" t="s">
+      <c r="J5" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="19">
+      <c r="K5" s="17">
         <v>7</v>
       </c>
-      <c r="L5" s="18" t="s">
+      <c r="L5" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="M5" s="20">
+      <c r="M5" s="18">
         <v>6</v>
       </c>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
+      <c r="N5" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" s="22">
+        <v>8</v>
+      </c>
+      <c r="P5" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q5" s="20">
+        <v>6</v>
+      </c>
     </row>
     <row r="6" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="14"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="19" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="7" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="11"/>
+      <c r="B7" s="10"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="11"/>
+      <c r="D7" s="10"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="11"/>
+      <c r="F7" s="10"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="11"/>
+      <c r="H7" s="10"/>
       <c r="I7" s="3"/>
-      <c r="J7" s="11"/>
+      <c r="J7" s="10"/>
       <c r="K7" s="3"/>
-      <c r="L7" s="11"/>
+      <c r="L7" s="10"/>
       <c r="M7" s="3"/>
-      <c r="N7" s="11"/>
+      <c r="N7" s="10"/>
       <c r="O7" s="3"/>
-      <c r="P7" s="11"/>
+      <c r="P7" s="10"/>
     </row>
     <row r="8" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="11"/>
+      <c r="B8" s="10"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="11"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="11"/>
+      <c r="F8" s="10"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="11"/>
+      <c r="H8" s="10"/>
       <c r="I8" s="3"/>
-      <c r="J8" s="11"/>
+      <c r="J8" s="10"/>
       <c r="K8" s="3"/>
-      <c r="L8" s="11"/>
+      <c r="L8" s="10"/>
       <c r="M8" s="3"/>
-      <c r="N8" s="11"/>
+      <c r="N8" s="10"/>
       <c r="O8" s="3"/>
-      <c r="P8" s="11"/>
+      <c r="P8" s="10"/>
     </row>
     <row r="9" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="11"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="3"/>
-      <c r="D9" s="11"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="11"/>
+      <c r="F9" s="10"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="11"/>
+      <c r="H9" s="10"/>
       <c r="I9" s="3"/>
-      <c r="J9" s="11"/>
+      <c r="J9" s="10"/>
       <c r="K9" s="3"/>
-      <c r="L9" s="11"/>
+      <c r="L9" s="10"/>
       <c r="M9" s="3"/>
-      <c r="N9" s="11"/>
+      <c r="N9" s="10"/>
       <c r="O9" s="3"/>
-      <c r="P9" s="11"/>
+      <c r="P9" s="10"/>
     </row>
     <row r="10" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="11"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="11"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="11"/>
+      <c r="F10" s="10"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="11"/>
+      <c r="H10" s="10"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="11"/>
+      <c r="J10" s="10"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="11"/>
+      <c r="L10" s="10"/>
       <c r="M10" s="3"/>
-      <c r="N10" s="11"/>
+      <c r="N10" s="10"/>
       <c r="O10" s="3"/>
-      <c r="P10" s="11"/>
+      <c r="P10" s="10"/>
     </row>
     <row r="11" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="11"/>
+      <c r="B11" s="10"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="11"/>
+      <c r="D11" s="10"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="11"/>
+      <c r="F11" s="10"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="11"/>
+      <c r="H11" s="10"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="11"/>
+      <c r="J11" s="10"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="11"/>
+      <c r="L11" s="10"/>
       <c r="M11" s="3"/>
-      <c r="N11" s="11"/>
+      <c r="N11" s="10"/>
       <c r="O11" s="3"/>
-      <c r="P11" s="11"/>
+      <c r="P11" s="10"/>
     </row>
     <row r="12" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="11"/>
+      <c r="B12" s="10"/>
       <c r="C12" s="3"/>
-      <c r="D12" s="11"/>
+      <c r="D12" s="10"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="11"/>
+      <c r="F12" s="10"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="11"/>
+      <c r="H12" s="10"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="11"/>
+      <c r="J12" s="10"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="11"/>
+      <c r="L12" s="10"/>
       <c r="M12" s="3"/>
-      <c r="N12" s="11"/>
+      <c r="N12" s="10"/>
       <c r="O12" s="3"/>
-      <c r="P12" s="11"/>
+      <c r="P12" s="10"/>
     </row>
     <row r="13" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="11"/>
+      <c r="B13" s="10"/>
       <c r="C13" s="3"/>
-      <c r="D13" s="11"/>
+      <c r="D13" s="10"/>
       <c r="E13" s="3"/>
-      <c r="F13" s="11"/>
+      <c r="F13" s="10"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="11"/>
+      <c r="H13" s="10"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="11"/>
+      <c r="J13" s="10"/>
       <c r="K13" s="3"/>
-      <c r="L13" s="11"/>
+      <c r="L13" s="10"/>
       <c r="M13" s="3"/>
-      <c r="N13" s="11"/>
+      <c r="N13" s="10"/>
       <c r="O13" s="3"/>
-      <c r="P13" s="11"/>
+      <c r="P13" s="10"/>
     </row>
     <row r="14" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>